<commit_message>
Assets/data: update (audio + data + supabase)
</commit_message>
<xml_diff>
--- a/word-data/category.xlsx
+++ b/word-data/category.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -683,9 +683,29 @@
         <v>13</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>nba</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v>Knicks</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>